<commit_message>
Reach and Media Report: covers section, headline and tile edits
Adds covers sales and orders for both windows (report, chart, workbook
sheet and summary rows), renames the headline, removes the plays-per-day,
cost-per-ThruPlay and signups-who-buy tiles, the earlier-pulls section and
the sources footer.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_016YF8TBJLzm45dMH9YfcQrr
</commit_message>
<xml_diff>
--- a/diggerlid-ops-hub/deliverables/reach-media-report-2026-09-23/reach-media-report-2026-09-23.xlsx
+++ b/diggerlid-ops-hub/deliverables/reach-media-report-2026-09-23/reach-media-report-2026-09-23.xlsx
@@ -11,8 +11,9 @@
     <sheet name="Meta campaigns prev 12m" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="Meta campaigns last 12m" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="Grease products" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Email signups monthly" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="Sources and caveats" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Covers products" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Email signups monthly" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Sources and caveats" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -70,7 +71,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
@@ -81,6 +82,7 @@
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="4" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -446,7 +448,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F35"/>
+  <dimension ref="A1:F38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="46" customWidth="1" min="1" max="1"/>
@@ -727,7 +729,6 @@
           <t>Derived</t>
         </is>
       </c>
-      <c r="F11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -747,7 +748,6 @@
           <t>Derived</t>
         </is>
       </c>
-      <c r="F12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -767,7 +767,6 @@
           <t>Derived</t>
         </is>
       </c>
-      <c r="F13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -787,7 +786,6 @@
           <t>Derived</t>
         </is>
       </c>
-      <c r="F14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -807,7 +805,6 @@
           <t>Derived</t>
         </is>
       </c>
-      <c r="F15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
@@ -1073,7 +1070,6 @@
           <t>Derived</t>
         </is>
       </c>
-      <c r="F26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -1095,7 +1091,6 @@
           <t>Derived</t>
         </is>
       </c>
-      <c r="F27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -1117,7 +1112,6 @@
           <t>Derived</t>
         </is>
       </c>
-      <c r="F28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -1139,7 +1133,6 @@
           <t>Derived</t>
         </is>
       </c>
-      <c r="F29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
@@ -1208,29 +1201,29 @@
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
         <is>
-          <t>EMAIL DATABASE (Klaviyo)</t>
-        </is>
-      </c>
-      <c r="B33" s="2" t="inlineStr"/>
-      <c r="C33" s="2" t="inlineStr"/>
-      <c r="D33" s="3" t="inlineStr"/>
-      <c r="E33" s="2" t="inlineStr"/>
-      <c r="F33" s="2" t="inlineStr"/>
+          <t>COVERS (Shopify net sales, AUD ex GST; titles containing Cover or Enclosure; GWP rows excluded)</t>
+        </is>
+      </c>
+      <c r="B33" s="2" t="n"/>
+      <c r="C33" s="2" t="n"/>
+      <c r="D33" s="2" t="n"/>
+      <c r="E33" s="2" t="n"/>
+      <c r="F33" s="2" t="n"/>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>New profiles added (Oct to Sep)</t>
+          <t>Covers net sales (8 products)</t>
         </is>
       </c>
       <c r="B34" s="4" t="n">
-        <v>7670</v>
+        <v>1135969.29</v>
       </c>
       <c r="C34" s="4" t="n">
-        <v>26186</v>
+        <v>1402609.8</v>
       </c>
       <c r="D34" s="5" t="n">
-        <v>2.414080834419817</v>
+        <v>0.2347251042323513</v>
       </c>
       <c r="E34" t="inlineStr">
         <is>
@@ -1239,31 +1232,95 @@
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>diggerlid-mer /api/emails monthly; Sep 2026 to the 22nd</t>
+          <t>ShopifyQL, same 12-month windows</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
+          <t>Covers orders</t>
+        </is>
+      </c>
+      <c r="B35" s="4" t="n">
+        <v>3111</v>
+      </c>
+      <c r="C35" s="4" t="n">
+        <v>4462</v>
+      </c>
+      <c r="D35" s="5" t="n">
+        <v>0.4342655094824814</v>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>Verified</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>Excludes 198 gift-with-purchase cover orders at $0 in the last window</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="2" t="inlineStr">
+        <is>
+          <t>EMAIL DATABASE (Klaviyo)</t>
+        </is>
+      </c>
+      <c r="B36" s="2" t="inlineStr"/>
+      <c r="C36" s="2" t="inlineStr"/>
+      <c r="D36" s="3" t="inlineStr"/>
+      <c r="E36" s="2" t="inlineStr"/>
+      <c r="F36" s="2" t="inlineStr"/>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>New profiles added (Oct to Sep)</t>
+        </is>
+      </c>
+      <c r="B37" s="4" t="n">
+        <v>7670</v>
+      </c>
+      <c r="C37" s="4" t="n">
+        <v>26186</v>
+      </c>
+      <c r="D37" s="5" t="n">
+        <v>2.414080834419817</v>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>Verified</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>diggerlid-mer /api/emails monthly; Sep 2026 to the 22nd</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
           <t>Of which Alia popup signups</t>
         </is>
       </c>
-      <c r="B35" s="4" t="n">
+      <c r="B38" s="4" t="n">
         <v>680</v>
       </c>
-      <c r="C35" s="4" t="n">
+      <c r="C38" s="4" t="n">
         <v>15317</v>
       </c>
-      <c r="D35" s="5" t="n">
+      <c r="D38" s="5" t="n">
         <v>21.525</v>
       </c>
-      <c r="E35" t="inlineStr">
+      <c r="E38" t="inlineStr">
         <is>
           <t>Verified</t>
         </is>
       </c>
-      <c r="F35" t="inlineStr">
+      <c r="F38" t="inlineStr">
         <is>
           <t>Alia popup live from Oct 2025</t>
         </is>
@@ -4271,6 +4328,308 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:G11"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="40" customWidth="1" min="1" max="1"/>
+    <col width="16" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="8" t="inlineStr">
+        <is>
+          <t>Product</t>
+        </is>
+      </c>
+      <c r="B1" s="8" t="inlineStr">
+        <is>
+          <t>Prev net sales</t>
+        </is>
+      </c>
+      <c r="C1" s="8" t="inlineStr">
+        <is>
+          <t>Prev orders</t>
+        </is>
+      </c>
+      <c r="D1" s="8" t="inlineStr">
+        <is>
+          <t>Last net sales</t>
+        </is>
+      </c>
+      <c r="E1" s="8" t="inlineStr">
+        <is>
+          <t>Last orders</t>
+        </is>
+      </c>
+      <c r="F1" s="8" t="inlineStr">
+        <is>
+          <t>Sales change</t>
+        </is>
+      </c>
+      <c r="G1" s="8" t="inlineStr">
+        <is>
+          <t>Orders change</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Pro Excavator Enclosure</t>
+        </is>
+      </c>
+      <c r="B2" s="4" t="n">
+        <v>698675.8100000001</v>
+      </c>
+      <c r="C2" t="n">
+        <v>1102</v>
+      </c>
+      <c r="D2" s="4" t="n">
+        <v>787145.97</v>
+      </c>
+      <c r="E2" t="n">
+        <v>1285</v>
+      </c>
+      <c r="F2" s="5" t="n">
+        <v>0.126625480278185</v>
+      </c>
+      <c r="G2" s="5" t="n">
+        <v>0.1660617059891107</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>1.7 Tonne Excavator Cover</t>
+        </is>
+      </c>
+      <c r="B3" s="4" t="n">
+        <v>202097.12</v>
+      </c>
+      <c r="C3" t="n">
+        <v>563</v>
+      </c>
+      <c r="D3" s="4" t="n">
+        <v>225085.74</v>
+      </c>
+      <c r="E3" t="n">
+        <v>668</v>
+      </c>
+      <c r="F3" s="5" t="n">
+        <v>0.1137503592332241</v>
+      </c>
+      <c r="G3" s="5" t="n">
+        <v>0.1865008880994672</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Draw Bar Cover</t>
+        </is>
+      </c>
+      <c r="B4" s="4" t="n">
+        <v>10995.3</v>
+      </c>
+      <c r="C4" t="n">
+        <v>79</v>
+      </c>
+      <c r="D4" s="4" t="n">
+        <v>107541.15</v>
+      </c>
+      <c r="E4" t="n">
+        <v>865</v>
+      </c>
+      <c r="F4" s="5" t="n">
+        <v>8.780647185615672</v>
+      </c>
+      <c r="G4" s="5" t="n">
+        <v>9.949367088607595</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Quicky Cover</t>
+        </is>
+      </c>
+      <c r="B5" s="4" t="n">
+        <v>82253.36</v>
+      </c>
+      <c r="C5" t="n">
+        <v>716</v>
+      </c>
+      <c r="D5" s="4" t="n">
+        <v>104884.56</v>
+      </c>
+      <c r="E5" t="n">
+        <v>866</v>
+      </c>
+      <c r="F5" s="5" t="n">
+        <v>0.2751401280142234</v>
+      </c>
+      <c r="G5" s="5" t="n">
+        <v>0.2094972067039107</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Mini Loader Cover</t>
+        </is>
+      </c>
+      <c r="B6" s="4" t="n">
+        <v>51220.28</v>
+      </c>
+      <c r="C6" t="n">
+        <v>203</v>
+      </c>
+      <c r="D6" s="4" t="n">
+        <v>65097.64</v>
+      </c>
+      <c r="E6" t="n">
+        <v>269</v>
+      </c>
+      <c r="F6" s="5" t="n">
+        <v>0.2709348718905871</v>
+      </c>
+      <c r="G6" s="5" t="n">
+        <v>0.3251231527093597</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Universal / Engine Covers</t>
+        </is>
+      </c>
+      <c r="B7" s="4" t="n">
+        <v>41044.79</v>
+      </c>
+      <c r="C7" t="n">
+        <v>311</v>
+      </c>
+      <c r="D7" s="4" t="n">
+        <v>53165.09</v>
+      </c>
+      <c r="E7" t="n">
+        <v>342</v>
+      </c>
+      <c r="F7" s="5" t="n">
+        <v>0.295294481954957</v>
+      </c>
+      <c r="G7" s="5" t="n">
+        <v>0.09967845659163976</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Skid Steer Loader Cover</t>
+        </is>
+      </c>
+      <c r="B8" s="4" t="n">
+        <v>31626.92</v>
+      </c>
+      <c r="C8" t="n">
+        <v>68</v>
+      </c>
+      <c r="D8" s="4" t="n">
+        <v>35249.94</v>
+      </c>
+      <c r="E8" t="n">
+        <v>81</v>
+      </c>
+      <c r="F8" s="5" t="n">
+        <v>0.1145549424351155</v>
+      </c>
+      <c r="G8" s="5" t="n">
+        <v>0.1911764705882353</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Micro Excavator Cover</t>
+        </is>
+      </c>
+      <c r="B9" s="4" t="n">
+        <v>18055.71</v>
+      </c>
+      <c r="C9" t="n">
+        <v>69</v>
+      </c>
+      <c r="D9" s="4" t="n">
+        <v>24439.71</v>
+      </c>
+      <c r="E9" t="n">
+        <v>86</v>
+      </c>
+      <c r="F9" s="5" t="n">
+        <v>0.353572360211811</v>
+      </c>
+      <c r="G9" s="5" t="n">
+        <v>0.2463768115942029</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Draw Bar Cover GWP (free gift)</t>
+        </is>
+      </c>
+      <c r="B10" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="C10" t="n">
+        <v>0</v>
+      </c>
+      <c r="D10" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="E10" t="n">
+        <v>102</v>
+      </c>
+      <c r="F10" s="5" t="n"/>
+      <c r="G10" s="5" t="n"/>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Universal / Engine Covers GWP (free gift)</t>
+        </is>
+      </c>
+      <c r="B11" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="C11" t="n">
+        <v>0</v>
+      </c>
+      <c r="D11" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="E11" t="n">
+        <v>96</v>
+      </c>
+      <c r="F11" s="5" t="n"/>
+      <c r="G11" s="5" t="n"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:E26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -4888,7 +5247,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>

<commit_message>
Reach and Media Report: monthly spend chart, state map, machine operators
Adds month-by-month Meta spend (chart and workbook sheet), an Australia
map of orders by billing state for both windows, and a machine-operators
section (grease plus covers) with orders growth; grease and covers reduced
to three points each.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_016YF8TBJLzm45dMH9YfcQrr
</commit_message>
<xml_diff>
--- a/diggerlid-ops-hub/deliverables/reach-media-report-2026-09-23/reach-media-report-2026-09-23.xlsx
+++ b/diggerlid-ops-hub/deliverables/reach-media-report-2026-09-23/reach-media-report-2026-09-23.xlsx
@@ -14,6 +14,9 @@
     <sheet name="Covers products" sheetId="5" state="visible" r:id="rId5"/>
     <sheet name="Email signups monthly" sheetId="6" state="visible" r:id="rId6"/>
     <sheet name="Sources and caveats" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="Meta spend monthly" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="AU orders by state" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="Machine operators" sheetId="10" state="visible" r:id="rId10"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -1331,6 +1334,155 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E6"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="52" customWidth="1" min="1" max="1"/>
+    <col width="18" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="70" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="8" t="inlineStr">
+        <is>
+          <t>Measure</t>
+        </is>
+      </c>
+      <c r="B1" s="8" t="inlineStr">
+        <is>
+          <t>Previous 12 months</t>
+        </is>
+      </c>
+      <c r="C1" s="8" t="inlineStr">
+        <is>
+          <t>Last 12 months</t>
+        </is>
+      </c>
+      <c r="D1" s="8" t="inlineStr">
+        <is>
+          <t>Change</t>
+        </is>
+      </c>
+      <c r="E1" s="8" t="inlineStr">
+        <is>
+          <t>Definition</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Operator orders (distinct orders containing grease or a cover)</t>
+        </is>
+      </c>
+      <c r="B2" s="4" t="n">
+        <v>7559</v>
+      </c>
+      <c r="C2" s="4" t="n">
+        <v>13359</v>
+      </c>
+      <c r="D2" s="5" t="n">
+        <v>0.767297261542532</v>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>ShopifyQL sales, product_title contains Cover, Enclosure, Grease or KAJO</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Operator net sales</t>
+        </is>
+      </c>
+      <c r="B3" s="4" t="n">
+        <v>2651251.13</v>
+      </c>
+      <c r="C3" s="4" t="n">
+        <v>3587495.23</v>
+      </c>
+      <c r="D3" s="5" t="n">
+        <v>0.3531329376557399</v>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>same filter, net sales ex GST</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Grease product orders (sum across 4 products)</t>
+        </is>
+      </c>
+      <c r="B4" s="4" t="n">
+        <v>8988</v>
+      </c>
+      <c r="C4" s="4" t="n">
+        <v>15396</v>
+      </c>
+      <c r="D4" s="5" t="n">
+        <v>0.7129506008010682</v>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>an order with two grease products counts twice</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Covers product orders (sum across 8 products, GWP excluded)</t>
+        </is>
+      </c>
+      <c r="B5" s="4" t="n">
+        <v>3111</v>
+      </c>
+      <c r="C5" s="4" t="n">
+        <v>4462</v>
+      </c>
+      <c r="D5" s="5" t="n">
+        <v>0.4342655094824814</v>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>same</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Total store net sales, last 12 months</t>
+        </is>
+      </c>
+      <c r="B6" s="4" t="n"/>
+      <c r="C6" s="4" t="n">
+        <v>4773555.86</v>
+      </c>
+      <c r="D6" s="5" t="n"/>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>all products; operator share 75%</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
@@ -5347,4 +5499,967 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F25"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="18" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="8" t="inlineStr">
+        <is>
+          <t>Month start</t>
+        </is>
+      </c>
+      <c r="B1" s="8" t="inlineStr">
+        <is>
+          <t>Month end</t>
+        </is>
+      </c>
+      <c r="C1" s="8" t="inlineStr">
+        <is>
+          <t>Spend (AUD)</t>
+        </is>
+      </c>
+      <c r="D1" s="8" t="inlineStr">
+        <is>
+          <t>Impressions</t>
+        </is>
+      </c>
+      <c r="E1" s="8" t="inlineStr">
+        <is>
+          <t>Attributed purchases</t>
+        </is>
+      </c>
+      <c r="F1" s="8" t="inlineStr">
+        <is>
+          <t>Window</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>2024-10-01</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>2024-10-31</t>
+        </is>
+      </c>
+      <c r="C2" s="4" t="n">
+        <v>46637</v>
+      </c>
+      <c r="D2" s="4" t="n">
+        <v>3932870</v>
+      </c>
+      <c r="E2" s="4" t="n">
+        <v>440</v>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>previous 12m</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>2024-11-01</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>2024-11-30</t>
+        </is>
+      </c>
+      <c r="C3" s="4" t="n">
+        <v>67262</v>
+      </c>
+      <c r="D3" s="4" t="n">
+        <v>4615068</v>
+      </c>
+      <c r="E3" s="4" t="n">
+        <v>673</v>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>previous 12m</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>2024-12-01</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>2024-12-31</t>
+        </is>
+      </c>
+      <c r="C4" s="4" t="n">
+        <v>72092</v>
+      </c>
+      <c r="D4" s="4" t="n">
+        <v>5450095</v>
+      </c>
+      <c r="E4" s="4" t="n">
+        <v>452</v>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>previous 12m</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>2025-01-01</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>2025-01-31</t>
+        </is>
+      </c>
+      <c r="C5" s="4" t="n">
+        <v>57480</v>
+      </c>
+      <c r="D5" s="4" t="n">
+        <v>5191739</v>
+      </c>
+      <c r="E5" s="4" t="n">
+        <v>406</v>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>previous 12m</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>2025-02-01</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>2025-02-28</t>
+        </is>
+      </c>
+      <c r="C6" s="4" t="n">
+        <v>58295</v>
+      </c>
+      <c r="D6" s="4" t="n">
+        <v>5128084</v>
+      </c>
+      <c r="E6" s="4" t="n">
+        <v>433</v>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>previous 12m</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>2025-03-01</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>2025-03-31</t>
+        </is>
+      </c>
+      <c r="C7" s="4" t="n">
+        <v>64744</v>
+      </c>
+      <c r="D7" s="4" t="n">
+        <v>5676536</v>
+      </c>
+      <c r="E7" s="4" t="n">
+        <v>462</v>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>previous 12m</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>2025-04-01</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>2025-04-30</t>
+        </is>
+      </c>
+      <c r="C8" s="4" t="n">
+        <v>61433</v>
+      </c>
+      <c r="D8" s="4" t="n">
+        <v>5354380</v>
+      </c>
+      <c r="E8" s="4" t="n">
+        <v>421</v>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>previous 12m</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>2025-05-01</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>2025-05-31</t>
+        </is>
+      </c>
+      <c r="C9" s="4" t="n">
+        <v>54969</v>
+      </c>
+      <c r="D9" s="4" t="n">
+        <v>4577642</v>
+      </c>
+      <c r="E9" s="4" t="n">
+        <v>519</v>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>previous 12m</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>2025-06-01</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>2025-06-30</t>
+        </is>
+      </c>
+      <c r="C10" s="4" t="n">
+        <v>91684</v>
+      </c>
+      <c r="D10" s="4" t="n">
+        <v>6891380</v>
+      </c>
+      <c r="E10" s="4" t="n">
+        <v>1038</v>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>previous 12m</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>2025-07-01</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>2025-07-31</t>
+        </is>
+      </c>
+      <c r="C11" s="4" t="n">
+        <v>91894</v>
+      </c>
+      <c r="D11" s="4" t="n">
+        <v>7352781</v>
+      </c>
+      <c r="E11" s="4" t="n">
+        <v>562</v>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>previous 12m</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>2025-08-01</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>2025-08-31</t>
+        </is>
+      </c>
+      <c r="C12" s="4" t="n">
+        <v>69395</v>
+      </c>
+      <c r="D12" s="4" t="n">
+        <v>5629782</v>
+      </c>
+      <c r="E12" s="4" t="n">
+        <v>541</v>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>previous 12m</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>2025-09-01</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>2025-09-30</t>
+        </is>
+      </c>
+      <c r="C13" s="4" t="n">
+        <v>58673</v>
+      </c>
+      <c r="D13" s="4" t="n">
+        <v>4865178</v>
+      </c>
+      <c r="E13" s="4" t="n">
+        <v>473</v>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>previous 12m</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>2025-10-01</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>2025-10-31</t>
+        </is>
+      </c>
+      <c r="C14" s="4" t="n">
+        <v>108109</v>
+      </c>
+      <c r="D14" s="4" t="n">
+        <v>10845552</v>
+      </c>
+      <c r="E14" s="4" t="n">
+        <v>852</v>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>last 12m</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>2025-11-01</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>2025-11-30</t>
+        </is>
+      </c>
+      <c r="C15" s="4" t="n">
+        <v>166140</v>
+      </c>
+      <c r="D15" s="4" t="n">
+        <v>13198004</v>
+      </c>
+      <c r="E15" s="4" t="n">
+        <v>1843</v>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>last 12m</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>2025-12-01</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>2025-12-31</t>
+        </is>
+      </c>
+      <c r="C16" s="4" t="n">
+        <v>94286</v>
+      </c>
+      <c r="D16" s="4" t="n">
+        <v>8235498</v>
+      </c>
+      <c r="E16" s="4" t="n">
+        <v>623</v>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>last 12m</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>2026-01-01</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>2026-01-31</t>
+        </is>
+      </c>
+      <c r="C17" s="4" t="n">
+        <v>48184</v>
+      </c>
+      <c r="D17" s="4" t="n">
+        <v>5770216</v>
+      </c>
+      <c r="E17" s="4" t="n">
+        <v>592</v>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>last 12m</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>2026-02-01</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>2026-02-28</t>
+        </is>
+      </c>
+      <c r="C18" s="4" t="n">
+        <v>84730</v>
+      </c>
+      <c r="D18" s="4" t="n">
+        <v>7960442</v>
+      </c>
+      <c r="E18" s="4" t="n">
+        <v>807</v>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>last 12m</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>2026-03-01</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>2026-03-31</t>
+        </is>
+      </c>
+      <c r="C19" s="4" t="n">
+        <v>100202</v>
+      </c>
+      <c r="D19" s="4" t="n">
+        <v>8896064</v>
+      </c>
+      <c r="E19" s="4" t="n">
+        <v>823</v>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>last 12m</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>2026-04-01</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>2026-04-30</t>
+        </is>
+      </c>
+      <c r="C20" s="4" t="n">
+        <v>108317</v>
+      </c>
+      <c r="D20" s="4" t="n">
+        <v>10620227</v>
+      </c>
+      <c r="E20" s="4" t="n">
+        <v>824</v>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>last 12m</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>2026-05-01</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>2026-05-31</t>
+        </is>
+      </c>
+      <c r="C21" s="4" t="n">
+        <v>122931</v>
+      </c>
+      <c r="D21" s="4" t="n">
+        <v>11922744</v>
+      </c>
+      <c r="E21" s="4" t="n">
+        <v>1311</v>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>last 12m</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="C22" s="4" t="n">
+        <v>197656</v>
+      </c>
+      <c r="D22" s="4" t="n">
+        <v>14452921</v>
+      </c>
+      <c r="E22" s="4" t="n">
+        <v>2595</v>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>last 12m</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>2026-07-31</t>
+        </is>
+      </c>
+      <c r="C23" s="4" t="n">
+        <v>162325</v>
+      </c>
+      <c r="D23" s="4" t="n">
+        <v>13828430</v>
+      </c>
+      <c r="E23" s="4" t="n">
+        <v>1291</v>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>last 12m</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>2026-08-01</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="C24" s="4" t="n">
+        <v>156945</v>
+      </c>
+      <c r="D24" s="4" t="n">
+        <v>11575102</v>
+      </c>
+      <c r="E24" s="4" t="n">
+        <v>1319</v>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>last 12m</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="C25" s="4" t="n">
+        <v>107304</v>
+      </c>
+      <c r="D25" s="4" t="n">
+        <v>8188698</v>
+      </c>
+      <c r="E25" s="4" t="n">
+        <v>864</v>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>last 12m</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G10"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="30" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="8" t="inlineStr">
+        <is>
+          <t>State</t>
+        </is>
+      </c>
+      <c r="B1" s="8" t="inlineStr">
+        <is>
+          <t>Prev orders</t>
+        </is>
+      </c>
+      <c r="C1" s="8" t="inlineStr">
+        <is>
+          <t>Prev net sales</t>
+        </is>
+      </c>
+      <c r="D1" s="8" t="inlineStr">
+        <is>
+          <t>Last orders</t>
+        </is>
+      </c>
+      <c r="E1" s="8" t="inlineStr">
+        <is>
+          <t>Last net sales</t>
+        </is>
+      </c>
+      <c r="F1" s="8" t="inlineStr">
+        <is>
+          <t>Orders change</t>
+        </is>
+      </c>
+      <c r="G1" s="8" t="inlineStr">
+        <is>
+          <t>Sales change</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>New South Wales</t>
+        </is>
+      </c>
+      <c r="B2" s="4" t="n">
+        <v>2336</v>
+      </c>
+      <c r="C2" s="4" t="n">
+        <v>777678.95</v>
+      </c>
+      <c r="D2" s="4" t="n">
+        <v>4990</v>
+      </c>
+      <c r="E2" s="4" t="n">
+        <v>1271393.22</v>
+      </c>
+      <c r="F2" s="5" t="n">
+        <v>1.136130136986301</v>
+      </c>
+      <c r="G2" s="5" t="n">
+        <v>0.6348561575441898</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Queensland</t>
+        </is>
+      </c>
+      <c r="B3" s="4" t="n">
+        <v>1866</v>
+      </c>
+      <c r="C3" s="4" t="n">
+        <v>621453.4</v>
+      </c>
+      <c r="D3" s="4" t="n">
+        <v>4315</v>
+      </c>
+      <c r="E3" s="4" t="n">
+        <v>1134566.36</v>
+      </c>
+      <c r="F3" s="5" t="n">
+        <v>1.312433011789925</v>
+      </c>
+      <c r="G3" s="5" t="n">
+        <v>0.825666027412514</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Victoria</t>
+        </is>
+      </c>
+      <c r="B4" s="4" t="n">
+        <v>1580</v>
+      </c>
+      <c r="C4" s="4" t="n">
+        <v>513923.43</v>
+      </c>
+      <c r="D4" s="4" t="n">
+        <v>3367</v>
+      </c>
+      <c r="E4" s="4" t="n">
+        <v>835233.65</v>
+      </c>
+      <c r="F4" s="5" t="n">
+        <v>1.131012658227848</v>
+      </c>
+      <c r="G4" s="5" t="n">
+        <v>0.6252102964054393</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Western Australia</t>
+        </is>
+      </c>
+      <c r="B5" s="4" t="n">
+        <v>751</v>
+      </c>
+      <c r="C5" s="4" t="n">
+        <v>272753.04</v>
+      </c>
+      <c r="D5" s="4" t="n">
+        <v>1904</v>
+      </c>
+      <c r="E5" s="4" t="n">
+        <v>530212.74</v>
+      </c>
+      <c r="F5" s="5" t="n">
+        <v>1.535286284953395</v>
+      </c>
+      <c r="G5" s="5" t="n">
+        <v>0.9439297175202888</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>South Australia</t>
+        </is>
+      </c>
+      <c r="B6" s="4" t="n">
+        <v>454</v>
+      </c>
+      <c r="C6" s="4" t="n">
+        <v>139356.45</v>
+      </c>
+      <c r="D6" s="4" t="n">
+        <v>1166</v>
+      </c>
+      <c r="E6" s="4" t="n">
+        <v>311484.72</v>
+      </c>
+      <c r="F6" s="5" t="n">
+        <v>1.568281938325991</v>
+      </c>
+      <c r="G6" s="5" t="n">
+        <v>1.235165433677451</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Tasmania</t>
+        </is>
+      </c>
+      <c r="B7" s="4" t="n">
+        <v>207</v>
+      </c>
+      <c r="C7" s="4" t="n">
+        <v>77360.49000000001</v>
+      </c>
+      <c r="D7" s="4" t="n">
+        <v>444</v>
+      </c>
+      <c r="E7" s="4" t="n">
+        <v>132466.7</v>
+      </c>
+      <c r="F7" s="5" t="n">
+        <v>1.144927536231884</v>
+      </c>
+      <c r="G7" s="5" t="n">
+        <v>0.7123301571642062</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Australian Capital Territory</t>
+        </is>
+      </c>
+      <c r="B8" s="4" t="n">
+        <v>76</v>
+      </c>
+      <c r="C8" s="4" t="n">
+        <v>21778.62</v>
+      </c>
+      <c r="D8" s="4" t="n">
+        <v>182</v>
+      </c>
+      <c r="E8" s="4" t="n">
+        <v>46284.51</v>
+      </c>
+      <c r="F8" s="5" t="n">
+        <v>1.394736842105263</v>
+      </c>
+      <c r="G8" s="5" t="n">
+        <v>1.125226942753949</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Northern Territory</t>
+        </is>
+      </c>
+      <c r="B9" s="4" t="n">
+        <v>37</v>
+      </c>
+      <c r="C9" s="4" t="n">
+        <v>10801.25</v>
+      </c>
+      <c r="D9" s="4" t="n">
+        <v>126</v>
+      </c>
+      <c r="E9" s="4" t="n">
+        <v>39389.29</v>
+      </c>
+      <c r="F9" s="5" t="n">
+        <v>2.405405405405405</v>
+      </c>
+      <c r="G9" s="5" t="n">
+        <v>2.646734405740077</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Australia total</t>
+        </is>
+      </c>
+      <c r="B10" s="4" t="n">
+        <v>7307</v>
+      </c>
+      <c r="C10" s="4" t="n">
+        <v>2435105.63</v>
+      </c>
+      <c r="D10" s="4" t="n">
+        <v>16495</v>
+      </c>
+      <c r="E10" s="4" t="n">
+        <v>4302234.83</v>
+      </c>
+      <c r="F10" s="5" t="n">
+        <v>1.25742438757356</v>
+      </c>
+      <c r="G10" s="5" t="n">
+        <v>0.7667549107510381</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Reach and Media Report: grease growth tile, email list size
Top tiles show grease as a percentage increase and the full Klaviyo list
size (44,804, up 141%) with the year's additions; list size added to the
growth chart, the email section and the workbook summary.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_016YF8TBJLzm45dMH9YfcQrr
</commit_message>
<xml_diff>
--- a/diggerlid-ops-hub/deliverables/reach-media-report-2026-09-23/reach-media-report-2026-09-23.xlsx
+++ b/diggerlid-ops-hub/deliverables/reach-media-report-2026-09-23/reach-media-report-2026-09-23.xlsx
@@ -451,7 +451,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F38"/>
+  <dimension ref="A1:F39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="46" customWidth="1" min="1" max="1"/>
@@ -1280,17 +1280,17 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>New profiles added (Oct to Sep)</t>
+          <t>Email list size (all Klaviyo profiles) at end of window</t>
         </is>
       </c>
       <c r="B37" s="4" t="n">
-        <v>7670</v>
+        <v>18618</v>
       </c>
       <c r="C37" s="4" t="n">
-        <v>26186</v>
+        <v>44804</v>
       </c>
       <c r="D37" s="5" t="n">
-        <v>2.414080834419817</v>
+        <v>1.406488344612741</v>
       </c>
       <c r="E37" t="inlineStr">
         <is>
@@ -1299,31 +1299,57 @@
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>diggerlid-mer /api/emails monthly; Sep 2026 to the 22nd</t>
+          <t>Profiles created before Oct 2024: 10,948 (yearly windows); plus each window's new profiles</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
+          <t>New profiles added (Oct to Sep)</t>
+        </is>
+      </c>
+      <c r="B38" s="4" t="n">
+        <v>7670</v>
+      </c>
+      <c r="C38" s="4" t="n">
+        <v>26186</v>
+      </c>
+      <c r="D38" s="5" t="n">
+        <v>2.414080834419817</v>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>Verified</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>diggerlid-mer /api/emails monthly; Sep 2026 to the 22nd</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
           <t>Of which Alia popup signups</t>
         </is>
       </c>
-      <c r="B38" s="4" t="n">
+      <c r="B39" s="4" t="n">
         <v>680</v>
       </c>
-      <c r="C38" s="4" t="n">
+      <c r="C39" s="4" t="n">
         <v>15317</v>
       </c>
-      <c r="D38" s="5" t="n">
+      <c r="D39" s="5" t="n">
         <v>21.525</v>
       </c>
-      <c r="E38" t="inlineStr">
+      <c r="E39" t="inlineStr">
         <is>
           <t>Verified</t>
         </is>
       </c>
-      <c r="F38" t="inlineStr">
+      <c r="F39" t="inlineStr">
         <is>
           <t>Alia popup live from Oct 2025</t>
         </is>

</xml_diff>

<commit_message>
Reach and Media Report: real state outlines, video watch-through, three efficiency tiles
Map now uses simplified public state boundary data; video section is a
two-chart watch-through deep dive (share of impressions and of plays per
milestone) with highlight stats beneath; efficiency tiles cut to three.
Workbook gains a video watch-through sheet.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_016YF8TBJLzm45dMH9YfcQrr
</commit_message>
<xml_diff>
--- a/diggerlid-ops-hub/deliverables/reach-media-report-2026-09-23/reach-media-report-2026-09-23.xlsx
+++ b/diggerlid-ops-hub/deliverables/reach-media-report-2026-09-23/reach-media-report-2026-09-23.xlsx
@@ -17,6 +17,7 @@
     <sheet name="Meta spend monthly" sheetId="8" state="visible" r:id="rId8"/>
     <sheet name="AU orders by state" sheetId="9" state="visible" r:id="rId9"/>
     <sheet name="Machine operators" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="Video watch-through" sheetId="11" state="visible" r:id="rId11"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -74,7 +75,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
@@ -86,6 +87,7 @@
     <xf numFmtId="4" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="10" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -1509,6 +1511,282 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:H8"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="28" customWidth="1" min="1" max="1"/>
+    <col width="16" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="60" customWidth="1" min="8" max="8"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="8" t="inlineStr">
+        <is>
+          <t>Milestone</t>
+        </is>
+      </c>
+      <c r="B1" s="8" t="inlineStr">
+        <is>
+          <t>Prev 12m count</t>
+        </is>
+      </c>
+      <c r="C1" s="8" t="inlineStr">
+        <is>
+          <t>Last 12m count</t>
+        </is>
+      </c>
+      <c r="D1" s="8" t="inlineStr">
+        <is>
+          <t>Prev % of impressions</t>
+        </is>
+      </c>
+      <c r="E1" s="8" t="inlineStr">
+        <is>
+          <t>Last % of impressions</t>
+        </is>
+      </c>
+      <c r="F1" s="8" t="inlineStr">
+        <is>
+          <t>Prev % of plays</t>
+        </is>
+      </c>
+      <c r="G1" s="8" t="inlineStr">
+        <is>
+          <t>Last % of plays</t>
+        </is>
+      </c>
+      <c r="H1" s="8" t="inlineStr">
+        <is>
+          <t>Source</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Impressions</t>
+        </is>
+      </c>
+      <c r="B2" s="4" t="n">
+        <v>64541983</v>
+      </c>
+      <c r="C2" s="4" t="n">
+        <v>126846504</v>
+      </c>
+      <c r="D2" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="E2" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="F2" s="9" t="n">
+        <v>2.435546528301887</v>
+      </c>
+      <c r="G2" s="9" t="n">
+        <v>1.766664401114206</v>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>Ads Manager pull 23 Sep 2026; 25% rows derived from quoted share of impressions</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Video plays (3s)</t>
+        </is>
+      </c>
+      <c r="B3" s="4" t="n">
+        <v>26500000</v>
+      </c>
+      <c r="C3" s="4" t="n">
+        <v>71800000</v>
+      </c>
+      <c r="D3" s="9" t="n">
+        <v>0.4105854634184388</v>
+      </c>
+      <c r="E3" s="9" t="n">
+        <v>0.5660384617300923</v>
+      </c>
+      <c r="F3" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="G3" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>Ads Manager pull 23 Sep 2026; 25% rows derived from quoted share of impressions</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Watched 25%</t>
+        </is>
+      </c>
+      <c r="B4" s="4" t="n">
+        <v>2775305</v>
+      </c>
+      <c r="C4" s="4" t="n">
+        <v>9386641</v>
+      </c>
+      <c r="D4" s="9" t="n">
+        <v>0.0429999958321702</v>
+      </c>
+      <c r="E4" s="9" t="n">
+        <v>0.07399999766647096</v>
+      </c>
+      <c r="F4" s="9" t="n">
+        <v>0.1047284905660377</v>
+      </c>
+      <c r="G4" s="9" t="n">
+        <v>0.1307331615598886</v>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>Ads Manager pull 23 Sep 2026; 25% rows derived from quoted share of impressions</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>ThruPlay (15s or complete)</t>
+        </is>
+      </c>
+      <c r="B5" s="4" t="n">
+        <v>1850000</v>
+      </c>
+      <c r="C5" s="4" t="n">
+        <v>4850000</v>
+      </c>
+      <c r="D5" s="9" t="n">
+        <v>0.02866351348392875</v>
+      </c>
+      <c r="E5" s="9" t="n">
+        <v>0.03823518857090456</v>
+      </c>
+      <c r="F5" s="9" t="n">
+        <v>0.06981132075471698</v>
+      </c>
+      <c r="G5" s="9" t="n">
+        <v>0.06754874651810584</v>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>Ads Manager pull 23 Sep 2026; 25% rows derived from quoted share of impressions</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Watched 50%</t>
+        </is>
+      </c>
+      <c r="B6" s="4" t="n">
+        <v>1360000</v>
+      </c>
+      <c r="C6" s="4" t="n">
+        <v>5010000</v>
+      </c>
+      <c r="D6" s="9" t="n">
+        <v>0.02107155585845573</v>
+      </c>
+      <c r="E6" s="9" t="n">
+        <v>0.03949655561654265</v>
+      </c>
+      <c r="F6" s="9" t="n">
+        <v>0.05132075471698113</v>
+      </c>
+      <c r="G6" s="9" t="n">
+        <v>0.06977715877437327</v>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>Ads Manager pull 23 Sep 2026; 25% rows derived from quoted share of impressions</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Watched 75%</t>
+        </is>
+      </c>
+      <c r="B7" s="4" t="n">
+        <v>846000</v>
+      </c>
+      <c r="C7" s="4" t="n">
+        <v>3240000</v>
+      </c>
+      <c r="D7" s="9" t="n">
+        <v>0.01310774724724525</v>
+      </c>
+      <c r="E7" s="9" t="n">
+        <v>0.0255426826741713</v>
+      </c>
+      <c r="F7" s="9" t="n">
+        <v>0.03192452830188679</v>
+      </c>
+      <c r="G7" s="9" t="n">
+        <v>0.04512534818941504</v>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>Ads Manager pull 23 Sep 2026; 25% rows derived from quoted share of impressions</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Watched 100%</t>
+        </is>
+      </c>
+      <c r="B8" s="4" t="n">
+        <v>307000</v>
+      </c>
+      <c r="C8" s="4" t="n">
+        <v>1100000</v>
+      </c>
+      <c r="D8" s="9" t="n">
+        <v>0.004756593859224932</v>
+      </c>
+      <c r="E8" s="9" t="n">
+        <v>0.008671898438761859</v>
+      </c>
+      <c r="F8" s="9" t="n">
+        <v>0.01158490566037736</v>
+      </c>
+      <c r="G8" s="9" t="n">
+        <v>0.01532033426183844</v>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>Ads Manager pull 23 Sep 2026; 25% rows derived from quoted share of impressions</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>